<commit_message>
nato aug barrel stats + new aug barrel pretty names
- added stats for nato aug barrels. the initial motivation for their addition in the first place was aesthetic appeal so their stats reflect that. they each have +0.05 dev to compensate for the now missing rat worx adapter, but they also have the upside of not needing the adapter's additional weight
- new pretty names for each standard aug barrel
- fixed "Löwenhurz" misspelling on HBAR barrel
-"556_barrels" updated
</commit_message>
<xml_diff>
--- a/changes/556-barrels.xlsx
+++ b/changes/556-barrels.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-dev\deadline-balancing\changes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whyth\Documents\GitHub\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03241501-FB71-4EA0-B7D9-DEA88ACF3463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11D4EBDB-C5BE-4EFF-926B-F47ED878103A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="m4-barrels" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="98">
   <si>
     <t>new</t>
   </si>
@@ -257,33 +257,18 @@
     <t>lowenhurz_aug_hbar_620mm_heavy_barrel</t>
   </si>
   <si>
-    <t>Löwenhurz AUG HBAR 620mm</t>
-  </si>
-  <si>
     <t>steyr_aug_508mm_barrel</t>
   </si>
   <si>
-    <t>Löwenherz AUG A3 5.56x45 508mm</t>
-  </si>
-  <si>
     <t>steyr_aug_457mm_barrel</t>
   </si>
   <si>
-    <t>Löwenherz AUG A3 5.56x45 457mm</t>
-  </si>
-  <si>
     <t>steyr_aug_407mm_barrel</t>
   </si>
   <si>
-    <t>Löwenherz AUG A3 5.56x45 407mm</t>
-  </si>
-  <si>
     <t>steyr_aug_350mm_barrel</t>
   </si>
   <si>
-    <t>Löwenherz AUG A3 5.56x45 350mm</t>
-  </si>
-  <si>
     <t>aft_mk_16_457mm_barrel</t>
   </si>
   <si>
@@ -300,6 +285,48 @@
   </si>
   <si>
     <t>AFT MK-16 254mm</t>
+  </si>
+  <si>
+    <t>steyr_aug_nato_350mm_barrel</t>
+  </si>
+  <si>
+    <t>Löwenherz AUG A3 NATO 5.56x45 350mm</t>
+  </si>
+  <si>
+    <t>steyr_aug_nato_407mm_barrel</t>
+  </si>
+  <si>
+    <t>Löwenherz AUG A3 NATO 5.56x45 407mm</t>
+  </si>
+  <si>
+    <t>steyr_aug_nato_457mm_barrel</t>
+  </si>
+  <si>
+    <t>Löwenherz AUG A3 NATO 5.56x45 457mm</t>
+  </si>
+  <si>
+    <t>steyr_aug_nato_508mm_barrel</t>
+  </si>
+  <si>
+    <t>Löwenherz AUG A3 NATO 5.56x45 508mm</t>
+  </si>
+  <si>
+    <t>Löwenherz AUG HBAR 620mm</t>
+  </si>
+  <si>
+    <t>Löwenherz AUG A3 Standard 5.56x45 350mm</t>
+  </si>
+  <si>
+    <t>Löwenherz AUG A3 Standard 5.56x45 407mm</t>
+  </si>
+  <si>
+    <t>Löwenherz AUG A3 Standard 5.56x45 457mm</t>
+  </si>
+  <si>
+    <t>Löwenherz AUG A3 Standard 5.56x45 508mm</t>
+  </si>
+  <si>
+    <t>muzzle_loudness</t>
   </si>
 </sst>
 </file>
@@ -659,20 +686,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA46"/>
+  <dimension ref="A1:AB50"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.42578125" customWidth="1"/>
     <col min="2" max="2" width="27.140625" customWidth="1"/>
-    <col min="3" max="25" width="6.7109375" customWidth="1"/>
+    <col min="3" max="26" width="6.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -710,37 +737,40 @@
         <v>12</v>
       </c>
       <c r="M2" t="s">
+        <v>97</v>
+      </c>
+      <c r="N2" t="s">
         <v>13</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>14</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>16</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>17</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>18</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>19</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" t="s">
         <v>20</v>
       </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
         <v>21</v>
       </c>
-      <c r="X2" t="s">
+      <c r="Y2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -771,46 +801,46 @@
       <c r="L3">
         <v>-0.06</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>5000</v>
       </c>
-      <c r="N3">
-        <f t="shared" ref="N3:N39" si="0">C3-D3*20-E3*0.8-F3*0.6-H3*5+I3*15+J3/300</f>
-        <v>-2.0266666666666655</v>
-      </c>
-      <c r="P3">
+      <c r="O3">
+        <f>C3-D3*20-E3*0.8-F3*0.6-H3*10+I3*15+J3/200-M3*5</f>
+        <v>1.0000000000002007E-2</v>
+      </c>
+      <c r="Q3">
         <v>0.18</v>
       </c>
-      <c r="Q3">
+      <c r="R3">
         <v>24</v>
       </c>
-      <c r="R3">
-        <v>0</v>
-      </c>
       <c r="S3">
-        <f t="shared" ref="S3:S17" si="1">ROUND(Q3*0.035+P3+R3, 2)</f>
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <f t="shared" ref="T3:T17" si="0">ROUND(R3*0.035+Q3+S3, 2)</f>
         <v>1.02</v>
       </c>
-      <c r="T3" s="1">
+      <c r="U3" s="1">
         <v>0.04</v>
       </c>
-      <c r="U3">
-        <f t="shared" ref="U3:U38" si="2">0.06+0.037*Q3+T3+R3</f>
+      <c r="V3">
+        <f t="shared" ref="V3:V42" si="1">0.06+0.037*R3+U3+S3</f>
         <v>0.98799999999999999</v>
       </c>
-      <c r="V3">
-        <f t="shared" ref="V3:V38" si="3">0+(Q3-14.5)*-0.043</f>
+      <c r="W3">
+        <f t="shared" ref="W3:W42" si="2">0+(R3-14.5)*-0.043</f>
         <v>-0.40849999999999997</v>
       </c>
-      <c r="X3">
+      <c r="Y3">
         <v>349.95</v>
       </c>
-      <c r="Y3">
-        <f t="shared" ref="Y3:Y10" si="4">X3*6</f>
+      <c r="Z3">
+        <f t="shared" ref="Z3:Z10" si="3">Y3*6</f>
         <v>2099.6999999999998</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -841,47 +871,47 @@
       <c r="L4">
         <v>-0.06</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>1600</v>
       </c>
-      <c r="N4">
+      <c r="O4">
+        <f>C4-D4*20-E4*0.8-F4*0.6-H4*10+I4*15+J4/200-M4*5</f>
+        <v>-5.3550000000000004</v>
+      </c>
+      <c r="Q4">
+        <v>0.18</v>
+      </c>
+      <c r="R4">
+        <v>20</v>
+      </c>
+      <c r="T4">
         <f t="shared" si="0"/>
-        <v>-6.8533333333333344</v>
-      </c>
-      <c r="P4">
-        <v>0.18</v>
-      </c>
-      <c r="Q4">
-        <v>20</v>
-      </c>
-      <c r="S4">
-        <f t="shared" si="1"/>
         <v>0.88</v>
       </c>
-      <c r="T4">
+      <c r="U4">
         <v>0.04</v>
       </c>
-      <c r="U4">
-        <f t="shared" si="2"/>
+      <c r="V4">
+        <f t="shared" si="1"/>
         <v>0.84000000000000008</v>
       </c>
-      <c r="V4">
+      <c r="W4">
+        <f t="shared" si="2"/>
+        <v>-0.23649999999999999</v>
+      </c>
+      <c r="Y4">
+        <v>344.99</v>
+      </c>
+      <c r="Z4">
         <f t="shared" si="3"/>
-        <v>-0.23649999999999999</v>
-      </c>
-      <c r="X4">
-        <v>344.99</v>
-      </c>
-      <c r="Y4">
-        <f t="shared" si="4"/>
         <v>2069.94</v>
       </c>
-      <c r="AA4">
-        <f>S7/S4</f>
+      <c r="AB4">
+        <f>T7/T4</f>
         <v>0.80681818181818177</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -912,46 +942,46 @@
       <c r="L5">
         <v>-0.06</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>2000</v>
       </c>
-      <c r="N5">
+      <c r="O5">
+        <f>C5-D5*20-E5*0.8-F5*0.6-H5*10+I5*15+J5/200-M5*5</f>
+        <v>-5.6949999999999967</v>
+      </c>
+      <c r="Q5">
+        <v>0.18</v>
+      </c>
+      <c r="R5">
+        <v>20</v>
+      </c>
+      <c r="S5">
+        <v>0.1</v>
+      </c>
+      <c r="T5">
         <f t="shared" si="0"/>
-        <v>-7.1133333333333297</v>
-      </c>
-      <c r="P5">
-        <v>0.18</v>
-      </c>
-      <c r="Q5">
-        <v>20</v>
-      </c>
-      <c r="R5">
-        <v>0.1</v>
-      </c>
-      <c r="S5">
-        <f t="shared" si="1"/>
         <v>0.98</v>
       </c>
-      <c r="T5">
+      <c r="U5">
         <v>0.04</v>
       </c>
-      <c r="U5">
-        <f t="shared" si="2"/>
+      <c r="V5">
+        <f t="shared" si="1"/>
         <v>0.94000000000000006</v>
       </c>
-      <c r="V5">
+      <c r="W5">
+        <f t="shared" si="2"/>
+        <v>-0.23649999999999999</v>
+      </c>
+      <c r="Y5">
+        <v>349.99</v>
+      </c>
+      <c r="Z5">
         <f t="shared" si="3"/>
-        <v>-0.23649999999999999</v>
-      </c>
-      <c r="X5">
-        <v>349.99</v>
-      </c>
-      <c r="Y5">
-        <f t="shared" si="4"/>
         <v>2099.94</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -982,46 +1012,46 @@
       <c r="L6">
         <v>-0.03</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <v>1800</v>
       </c>
-      <c r="N6">
+      <c r="O6">
+        <f>C6-D6*20-E6*0.8-F6*0.6-H6*10+I6*15+J6/200-M6*5</f>
+        <v>-4.5950000000000006</v>
+      </c>
+      <c r="Q6">
+        <v>0.15</v>
+      </c>
+      <c r="R6">
+        <v>18</v>
+      </c>
+      <c r="S6">
+        <v>-0.04</v>
+      </c>
+      <c r="T6">
         <f t="shared" si="0"/>
-        <v>-5.4633333333333338</v>
-      </c>
-      <c r="P6">
-        <v>0.15</v>
-      </c>
-      <c r="Q6">
-        <v>18</v>
-      </c>
-      <c r="R6">
-        <v>-0.04</v>
-      </c>
-      <c r="S6">
-        <f t="shared" si="1"/>
         <v>0.74</v>
       </c>
-      <c r="T6">
+      <c r="U6">
         <v>0.03</v>
       </c>
-      <c r="U6">
-        <f t="shared" si="2"/>
+      <c r="V6">
+        <f t="shared" si="1"/>
         <v>0.71599999999999997</v>
       </c>
-      <c r="V6">
+      <c r="W6">
+        <f t="shared" si="2"/>
+        <v>-0.15049999999999999</v>
+      </c>
+      <c r="Y6">
+        <v>372</v>
+      </c>
+      <c r="Z6">
         <f t="shared" si="3"/>
-        <v>-0.15049999999999999</v>
-      </c>
-      <c r="X6">
-        <v>372</v>
-      </c>
-      <c r="Y6">
-        <f t="shared" si="4"/>
         <v>2232</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>31</v>
       </c>
@@ -1052,43 +1082,43 @@
       <c r="L7">
         <v>-0.03</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <v>1100</v>
       </c>
-      <c r="N7">
+      <c r="O7">
+        <f>C7-D7*20-E7*0.8-F7*0.6-H7*10+I7*15+J7/200-M7*5</f>
+        <v>-5.56</v>
+      </c>
+      <c r="Q7">
+        <v>0.15</v>
+      </c>
+      <c r="R7">
+        <v>16</v>
+      </c>
+      <c r="T7">
         <f t="shared" si="0"/>
-        <v>-5.9899999999999993</v>
-      </c>
-      <c r="P7">
-        <v>0.15</v>
-      </c>
-      <c r="Q7">
-        <v>16</v>
-      </c>
-      <c r="S7">
-        <f t="shared" si="1"/>
         <v>0.71</v>
       </c>
-      <c r="T7">
+      <c r="U7">
         <v>0.03</v>
       </c>
-      <c r="U7">
-        <f t="shared" si="2"/>
+      <c r="V7">
+        <f t="shared" si="1"/>
         <v>0.68199999999999994</v>
       </c>
-      <c r="V7">
+      <c r="W7">
+        <f t="shared" si="2"/>
+        <v>-6.4500000000000002E-2</v>
+      </c>
+      <c r="Y7">
+        <v>329.99</v>
+      </c>
+      <c r="Z7">
         <f t="shared" si="3"/>
-        <v>-6.4500000000000002E-2</v>
-      </c>
-      <c r="X7">
-        <v>329.99</v>
-      </c>
-      <c r="Y7">
-        <f t="shared" si="4"/>
         <v>1979.94</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -1116,46 +1146,46 @@
       <c r="J8">
         <v>78</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <v>1200</v>
       </c>
-      <c r="N8">
+      <c r="O8">
+        <f>C8-D8*20-E8*0.8-F8*0.6-H8*10+I8*15+J8/200-M8*5</f>
+        <v>-6.21</v>
+      </c>
+      <c r="Q8">
+        <v>0.12</v>
+      </c>
+      <c r="R8">
+        <v>16</v>
+      </c>
+      <c r="S8">
+        <v>0.04</v>
+      </c>
+      <c r="T8">
         <f t="shared" si="0"/>
-        <v>-6.6899999999999995</v>
-      </c>
-      <c r="P8">
-        <v>0.12</v>
-      </c>
-      <c r="Q8">
-        <v>16</v>
-      </c>
-      <c r="R8">
-        <v>0.04</v>
-      </c>
-      <c r="S8">
-        <f t="shared" si="1"/>
         <v>0.72</v>
       </c>
-      <c r="T8">
+      <c r="U8">
         <v>0.02</v>
       </c>
-      <c r="U8">
-        <f t="shared" si="2"/>
+      <c r="V8">
+        <f t="shared" si="1"/>
         <v>0.71199999999999997</v>
       </c>
-      <c r="V8">
+      <c r="W8">
+        <f t="shared" si="2"/>
+        <v>-6.4500000000000002E-2</v>
+      </c>
+      <c r="Y8">
+        <v>279.99</v>
+      </c>
+      <c r="Z8">
         <f t="shared" si="3"/>
-        <v>-6.4500000000000002E-2</v>
-      </c>
-      <c r="X8">
-        <v>279.99</v>
-      </c>
-      <c r="Y8">
-        <f t="shared" si="4"/>
         <v>1679.94</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -1183,46 +1213,46 @@
       <c r="J9">
         <v>45</v>
       </c>
-      <c r="M9">
+      <c r="N9">
         <v>800</v>
       </c>
-      <c r="N9">
+      <c r="O9">
+        <f>C9-D9*20-E9*0.8-F9*0.6-H9*10+I9*15+J9/200-M9*5</f>
+        <v>-5.9750000000000005</v>
+      </c>
+      <c r="Q9">
+        <v>0.12</v>
+      </c>
+      <c r="R9">
+        <v>14.5</v>
+      </c>
+      <c r="S9">
+        <v>0.04</v>
+      </c>
+      <c r="T9">
         <f t="shared" si="0"/>
-        <v>-6.15</v>
-      </c>
-      <c r="P9">
-        <v>0.12</v>
-      </c>
-      <c r="Q9">
-        <v>14.5</v>
-      </c>
-      <c r="R9">
-        <v>0.04</v>
-      </c>
-      <c r="S9">
-        <f t="shared" si="1"/>
         <v>0.67</v>
       </c>
-      <c r="T9">
+      <c r="U9">
         <v>0.02</v>
       </c>
-      <c r="U9">
-        <f t="shared" si="2"/>
+      <c r="V9">
+        <f t="shared" si="1"/>
         <v>0.65650000000000008</v>
       </c>
-      <c r="V9">
+      <c r="W9">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y9">
+        <v>349</v>
+      </c>
+      <c r="Z9">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="X9">
-        <v>349</v>
-      </c>
-      <c r="Y9">
-        <f t="shared" si="4"/>
         <v>2094</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>37</v>
       </c>
@@ -1250,40 +1280,40 @@
       <c r="J10">
         <v>33</v>
       </c>
-      <c r="M10">
-        <v>0</v>
-      </c>
       <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <f>C10-D10*20-E10*0.8-F10*0.6-H10*10+I10*15+J10/200-M10*5</f>
+        <v>-6.1349999999999998</v>
+      </c>
+      <c r="Q10">
+        <v>0.12</v>
+      </c>
+      <c r="R10">
+        <v>14.5</v>
+      </c>
+      <c r="T10">
         <f t="shared" si="0"/>
-        <v>-6.1899999999999995</v>
-      </c>
-      <c r="P10">
-        <v>0.12</v>
-      </c>
-      <c r="Q10">
-        <v>14.5</v>
-      </c>
-      <c r="S10">
-        <f t="shared" si="1"/>
         <v>0.63</v>
       </c>
-      <c r="T10">
+      <c r="U10">
         <v>0.02</v>
       </c>
-      <c r="U10">
-        <f t="shared" si="2"/>
+      <c r="V10">
+        <f t="shared" si="1"/>
         <v>0.61650000000000005</v>
       </c>
-      <c r="V10">
+      <c r="W10">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Z10">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="Y10">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>39</v>
       </c>
@@ -1314,39 +1344,39 @@
       <c r="L11">
         <v>-0.03</v>
       </c>
-      <c r="M11">
+      <c r="N11">
         <v>2000</v>
       </c>
-      <c r="N11">
+      <c r="O11">
+        <f>C11-D11*20-E11*0.8-F11*0.6-H11*10+I11*15+J11/200-M11*5</f>
+        <v>-5.665</v>
+      </c>
+      <c r="Q11">
+        <v>0.15</v>
+      </c>
+      <c r="R11">
+        <v>13.7</v>
+      </c>
+      <c r="S11">
+        <v>0.02</v>
+      </c>
+      <c r="T11">
         <f t="shared" si="0"/>
-        <v>-5.5266666666666664</v>
-      </c>
-      <c r="P11">
-        <v>0.15</v>
-      </c>
-      <c r="Q11">
-        <v>13.7</v>
-      </c>
-      <c r="R11">
-        <v>0.02</v>
-      </c>
-      <c r="S11">
-        <f t="shared" si="1"/>
         <v>0.65</v>
       </c>
-      <c r="T11">
+      <c r="U11">
         <v>0.03</v>
       </c>
-      <c r="U11">
-        <f t="shared" si="2"/>
+      <c r="V11">
+        <f t="shared" si="1"/>
         <v>0.6169</v>
       </c>
-      <c r="V11">
-        <f t="shared" si="3"/>
+      <c r="W11">
+        <f t="shared" si="2"/>
         <v>3.4400000000000028E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>41</v>
       </c>
@@ -1374,43 +1404,43 @@
       <c r="J12">
         <v>-34</v>
       </c>
-      <c r="M12">
+      <c r="N12">
         <v>1200</v>
       </c>
-      <c r="N12">
+      <c r="O12">
+        <f>C12-D12*20-E12*0.8-F12*0.6-H12*10+I12*15+J12/200-M12*5</f>
+        <v>-6.97</v>
+      </c>
+      <c r="Q12">
+        <v>0.12</v>
+      </c>
+      <c r="R12">
+        <v>12.5</v>
+      </c>
+      <c r="T12">
         <f t="shared" si="0"/>
-        <v>-6.4633333333333338</v>
-      </c>
-      <c r="P12">
-        <v>0.12</v>
-      </c>
-      <c r="Q12">
-        <v>12.5</v>
-      </c>
-      <c r="S12">
-        <f t="shared" si="1"/>
         <v>0.56000000000000005</v>
       </c>
-      <c r="T12">
+      <c r="U12">
         <v>0.02</v>
       </c>
-      <c r="U12">
-        <f t="shared" si="2"/>
+      <c r="V12">
+        <f t="shared" si="1"/>
         <v>0.54249999999999998</v>
       </c>
-      <c r="V12">
-        <f t="shared" si="3"/>
+      <c r="W12">
+        <f t="shared" si="2"/>
         <v>8.5999999999999993E-2</v>
       </c>
-      <c r="X12">
+      <c r="Y12">
         <v>338</v>
       </c>
-      <c r="Y12">
-        <f t="shared" ref="Y12:Y17" si="5">X12*6</f>
+      <c r="Z12">
+        <f t="shared" ref="Z12:Z17" si="4">Y12*6</f>
         <v>2028</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -1438,43 +1468,43 @@
       <c r="J13">
         <v>-72</v>
       </c>
-      <c r="M13">
+      <c r="N13">
         <v>1100</v>
       </c>
-      <c r="N13">
+      <c r="O13">
+        <f>C13-D13*20-E13*0.8-F13*0.6-H13*10+I13*15+J13/200-M13*5</f>
+        <v>-7.0100000000000007</v>
+      </c>
+      <c r="Q13">
+        <v>0.12</v>
+      </c>
+      <c r="R13">
+        <v>11.5</v>
+      </c>
+      <c r="T13">
         <f t="shared" si="0"/>
-        <v>-6.2400000000000011</v>
-      </c>
-      <c r="P13">
-        <v>0.12</v>
-      </c>
-      <c r="Q13">
-        <v>11.5</v>
-      </c>
-      <c r="S13">
-        <f t="shared" si="1"/>
         <v>0.52</v>
       </c>
-      <c r="T13">
+      <c r="U13">
         <v>0.02</v>
       </c>
-      <c r="U13">
-        <f t="shared" si="2"/>
+      <c r="V13">
+        <f t="shared" si="1"/>
         <v>0.50549999999999995</v>
       </c>
-      <c r="V13">
-        <f t="shared" si="3"/>
+      <c r="W13">
+        <f t="shared" si="2"/>
         <v>0.129</v>
       </c>
-      <c r="X13">
+      <c r="Y13">
         <v>155</v>
       </c>
-      <c r="Y13">
-        <f t="shared" si="5"/>
+      <c r="Z13">
+        <f t="shared" si="4"/>
         <v>930</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>45</v>
       </c>
@@ -1502,43 +1532,43 @@
       <c r="J14">
         <v>-113</v>
       </c>
-      <c r="M14">
+      <c r="N14">
         <v>1200</v>
       </c>
-      <c r="N14">
+      <c r="O14">
+        <f>C14-D14*20-E14*0.8-F14*0.6-H14*10+I14*15+J14/200-M14*5</f>
+        <v>-7.6649999999999991</v>
+      </c>
+      <c r="Q14">
+        <v>0.12</v>
+      </c>
+      <c r="R14">
+        <v>10.5</v>
+      </c>
+      <c r="T14">
         <f t="shared" si="0"/>
-        <v>-6.626666666666666</v>
-      </c>
-      <c r="P14">
-        <v>0.12</v>
-      </c>
-      <c r="Q14">
-        <v>10.5</v>
-      </c>
-      <c r="S14">
-        <f t="shared" si="1"/>
         <v>0.49</v>
       </c>
-      <c r="T14">
+      <c r="U14">
         <v>0.02</v>
       </c>
-      <c r="U14">
-        <f t="shared" si="2"/>
+      <c r="V14">
+        <f t="shared" si="1"/>
         <v>0.46849999999999997</v>
       </c>
-      <c r="V14">
-        <f t="shared" si="3"/>
+      <c r="W14">
+        <f t="shared" si="2"/>
         <v>0.17199999999999999</v>
       </c>
-      <c r="X14">
+      <c r="Y14">
         <v>299</v>
       </c>
-      <c r="Y14">
-        <f t="shared" si="5"/>
+      <c r="Z14">
+        <f t="shared" si="4"/>
         <v>1794</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>47</v>
       </c>
@@ -1569,40 +1599,40 @@
       <c r="L15">
         <v>0.03</v>
       </c>
-      <c r="M15">
+      <c r="N15">
         <v>1300</v>
       </c>
-      <c r="N15">
+      <c r="O15">
+        <f>C15-D15*20-E15*0.8-F15*0.6-H15*10+I15*15+J15/200-M15*5</f>
+        <v>-8.48</v>
+      </c>
+      <c r="Q15">
+        <v>0.09</v>
+      </c>
+      <c r="R15">
+        <v>7.5</v>
+      </c>
+      <c r="T15">
         <f t="shared" si="0"/>
-        <v>-6.5366666666666671</v>
-      </c>
-      <c r="P15">
-        <v>0.09</v>
-      </c>
-      <c r="Q15">
-        <v>7.5</v>
-      </c>
-      <c r="S15">
-        <f t="shared" si="1"/>
         <v>0.35</v>
       </c>
-      <c r="T15">
+      <c r="U15">
         <v>0.01</v>
       </c>
-      <c r="U15">
-        <f t="shared" si="2"/>
+      <c r="V15">
+        <f t="shared" si="1"/>
         <v>0.34749999999999998</v>
       </c>
-      <c r="V15">
-        <f t="shared" si="3"/>
+      <c r="W15">
+        <f t="shared" si="2"/>
         <v>0.30099999999999999</v>
       </c>
-      <c r="Y15">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Z15">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>49</v>
       </c>
@@ -1633,43 +1663,43 @@
       <c r="L16">
         <v>6.3E-2</v>
       </c>
-      <c r="M16">
+      <c r="N16">
         <v>1400</v>
       </c>
-      <c r="N16">
+      <c r="O16">
+        <f>C16-D16*20-E16*0.8-F16*0.6-H16*10+I16*15+J16/200-M16*5</f>
+        <v>-9.35</v>
+      </c>
+      <c r="Q16">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="R16">
+        <v>5</v>
+      </c>
+      <c r="T16">
         <f t="shared" si="0"/>
-        <v>-6.6</v>
-      </c>
-      <c r="P16">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="Q16">
-        <v>5</v>
-      </c>
-      <c r="S16">
-        <f t="shared" si="1"/>
         <v>0.25</v>
       </c>
-      <c r="T16">
-        <v>0</v>
-      </c>
       <c r="U16">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="V16">
+        <f t="shared" si="1"/>
         <v>0.245</v>
       </c>
-      <c r="V16">
-        <f t="shared" si="3"/>
+      <c r="W16">
+        <f t="shared" si="2"/>
         <v>0.40849999999999997</v>
       </c>
-      <c r="X16">
+      <c r="Y16">
         <v>149.94999999999999</v>
       </c>
-      <c r="Y16">
-        <f t="shared" si="5"/>
+      <c r="Z16">
+        <f t="shared" si="4"/>
         <v>899.69999999999993</v>
       </c>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>51</v>
       </c>
@@ -1700,57 +1730,53 @@
       <c r="L17">
         <v>0.125</v>
       </c>
-      <c r="M17">
+      <c r="N17">
         <v>2000</v>
       </c>
-      <c r="N17">
+      <c r="O17">
+        <f>C17-D17*20-E17*0.8-F17*0.6-H17*10+I17*15+J17/200-M17*5</f>
+        <v>-63.73</v>
+      </c>
+      <c r="Q17">
+        <v>0.05</v>
+      </c>
+      <c r="R17">
+        <v>2</v>
+      </c>
+      <c r="S17">
+        <v>-0.01</v>
+      </c>
+      <c r="T17">
         <f t="shared" si="0"/>
-        <v>-37.286666666666662</v>
-      </c>
-      <c r="P17">
-        <v>0.05</v>
-      </c>
-      <c r="Q17">
-        <v>2</v>
-      </c>
-      <c r="R17">
-        <v>-0.01</v>
-      </c>
-      <c r="S17">
-        <f t="shared" si="1"/>
         <v>0.11</v>
       </c>
-      <c r="T17">
-        <v>0</v>
-      </c>
       <c r="U17">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="V17">
+        <f t="shared" si="1"/>
         <v>0.12400000000000001</v>
       </c>
-      <c r="V17">
-        <f t="shared" si="3"/>
+      <c r="W17">
+        <f t="shared" si="2"/>
         <v>0.53749999999999998</v>
       </c>
-      <c r="Y17">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="N18">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="U18">
-        <f t="shared" si="2"/>
+      <c r="Z17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="V18">
+        <f t="shared" si="1"/>
         <v>0.06</v>
       </c>
-      <c r="V18">
-        <f t="shared" si="3"/>
+      <c r="W18">
+        <f t="shared" si="2"/>
         <v>0.62349999999999994</v>
       </c>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>53</v>
       </c>
@@ -1778,36 +1804,36 @@
       <c r="J19">
         <v>-140</v>
       </c>
-      <c r="M19">
+      <c r="N19">
         <v>1000</v>
       </c>
-      <c r="N19">
-        <f t="shared" si="0"/>
-        <v>-11.516666666666666</v>
-      </c>
-      <c r="P19">
+      <c r="O19">
+        <f>C19-D19*20-E19*0.8-F19*0.6-H19*10+I19*15+J19/200-M19*5</f>
+        <v>-12.95</v>
+      </c>
+      <c r="Q19">
         <v>0.04</v>
       </c>
-      <c r="Q19">
+      <c r="R19">
         <v>9</v>
       </c>
-      <c r="R19">
+      <c r="S19">
         <v>0.01</v>
       </c>
-      <c r="S19">
-        <f>ROUND(Q19*0.033+P19+R19, 2)</f>
+      <c r="T19">
+        <f>ROUND(R19*0.033+Q19+S19, 2)</f>
         <v>0.35</v>
       </c>
-      <c r="U19">
-        <f t="shared" si="2"/>
+      <c r="V19">
+        <f t="shared" si="1"/>
         <v>0.40299999999999997</v>
       </c>
-      <c r="V19">
-        <f t="shared" si="3"/>
+      <c r="W19">
+        <f t="shared" si="2"/>
         <v>0.23649999999999999</v>
       </c>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>55</v>
       </c>
@@ -1835,36 +1861,36 @@
       <c r="J20">
         <v>-100</v>
       </c>
-      <c r="M20">
+      <c r="N20">
         <v>1000</v>
       </c>
-      <c r="N20">
-        <f t="shared" si="0"/>
-        <v>-11.433333333333334</v>
-      </c>
-      <c r="P20">
+      <c r="O20">
+        <f>C20-D20*20-E20*0.8-F20*0.6-H20*10+I20*15+J20/200-M20*5</f>
+        <v>-12.5</v>
+      </c>
+      <c r="Q20">
         <v>0.04</v>
       </c>
-      <c r="Q20">
+      <c r="R20">
         <v>10.4</v>
       </c>
-      <c r="R20">
+      <c r="S20">
         <v>0.02</v>
       </c>
-      <c r="S20">
-        <f t="shared" ref="S20:S28" si="6">ROUND(Q20*0.033+P49+R20, 2)</f>
+      <c r="T20">
+        <f>ROUND(R20*0.033+Q53+S20, 2)</f>
         <v>0.36</v>
       </c>
-      <c r="U20">
-        <f t="shared" si="2"/>
+      <c r="V20">
+        <f t="shared" si="1"/>
         <v>0.46479999999999999</v>
       </c>
-      <c r="V20">
-        <f t="shared" si="3"/>
+      <c r="W20">
+        <f t="shared" si="2"/>
         <v>0.17629999999999996</v>
       </c>
     </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>57</v>
       </c>
@@ -1892,36 +1918,36 @@
       <c r="J21">
         <v>-80</v>
       </c>
-      <c r="M21">
+      <c r="N21">
         <v>1000</v>
       </c>
-      <c r="N21">
-        <f t="shared" si="0"/>
-        <v>-10.716666666666667</v>
-      </c>
-      <c r="P21">
+      <c r="O21">
+        <f>C21-D21*20-E21*0.8-F21*0.6-H21*10+I21*15+J21/200-M21*5</f>
+        <v>-11.6</v>
+      </c>
+      <c r="Q21">
         <v>0.04</v>
       </c>
-      <c r="Q21">
+      <c r="R21">
         <v>11</v>
       </c>
-      <c r="R21">
-        <v>0</v>
-      </c>
       <c r="S21">
-        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="T21">
+        <f>ROUND(R21*0.033+Q54+S21, 2)</f>
         <v>0.36</v>
       </c>
-      <c r="U21">
-        <f t="shared" si="2"/>
+      <c r="V21">
+        <f t="shared" si="1"/>
         <v>0.46699999999999997</v>
       </c>
-      <c r="V21">
-        <f t="shared" si="3"/>
+      <c r="W21">
+        <f t="shared" si="2"/>
         <v>0.15049999999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>59</v>
       </c>
@@ -1949,36 +1975,36 @@
       <c r="J22">
         <v>-30</v>
       </c>
-      <c r="M22">
+      <c r="N22">
         <v>1000</v>
       </c>
-      <c r="N22">
-        <f t="shared" si="0"/>
-        <v>-11.600000000000001</v>
-      </c>
-      <c r="P22">
+      <c r="O22">
+        <f>C22-D22*20-E22*0.8-F22*0.6-H22*10+I22*15+J22/200-M22*5</f>
+        <v>-12.050000000000002</v>
+      </c>
+      <c r="Q22">
         <v>0.04</v>
       </c>
-      <c r="Q22">
+      <c r="R22">
         <v>12.5</v>
       </c>
-      <c r="R22">
-        <v>0</v>
-      </c>
       <c r="S22">
-        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="T22">
+        <f>ROUND(R22*0.033+Q55+S22, 2)</f>
         <v>0.41</v>
       </c>
-      <c r="U22">
-        <f t="shared" si="2"/>
+      <c r="V22">
+        <f t="shared" si="1"/>
         <v>0.52249999999999996</v>
       </c>
-      <c r="V22">
-        <f t="shared" si="3"/>
+      <c r="W22">
+        <f t="shared" si="2"/>
         <v>8.5999999999999993E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>61</v>
       </c>
@@ -2006,36 +2032,36 @@
       <c r="J23">
         <v>50</v>
       </c>
-      <c r="M23">
-        <v>0</v>
-      </c>
       <c r="N23">
-        <f t="shared" si="0"/>
-        <v>-12.383333333333335</v>
-      </c>
-      <c r="P23">
+        <v>0</v>
+      </c>
+      <c r="O23">
+        <f>C23-D23*20-E23*0.8-F23*0.6-H23*10+I23*15+J23/200-M23*5</f>
+        <v>-12.3</v>
+      </c>
+      <c r="Q23">
         <v>0.04</v>
       </c>
-      <c r="Q23">
+      <c r="R23">
         <v>14.5</v>
       </c>
-      <c r="R23">
+      <c r="S23">
         <v>0.05</v>
       </c>
-      <c r="S23">
-        <f t="shared" si="6"/>
+      <c r="T23">
+        <f>ROUND(R23*0.033+Q56+S23, 2)</f>
         <v>0.53</v>
       </c>
-      <c r="U23">
-        <f t="shared" si="2"/>
+      <c r="V23">
+        <f t="shared" si="1"/>
         <v>0.64650000000000007</v>
       </c>
-      <c r="V23">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="W23">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>63</v>
       </c>
@@ -2063,36 +2089,36 @@
       <c r="J24">
         <v>50</v>
       </c>
-      <c r="M24">
-        <v>0</v>
-      </c>
       <c r="N24">
-        <f t="shared" si="0"/>
-        <v>-11.683333333333335</v>
-      </c>
-      <c r="P24">
+        <v>0</v>
+      </c>
+      <c r="O24">
+        <f>C24-D24*20-E24*0.8-F24*0.6-H24*10+I24*15+J24/200-M24*5</f>
+        <v>-11.500000000000002</v>
+      </c>
+      <c r="Q24">
         <v>0.04</v>
       </c>
-      <c r="Q24">
+      <c r="R24">
         <v>14.5</v>
       </c>
-      <c r="R24">
+      <c r="S24">
         <v>0.02</v>
       </c>
-      <c r="S24">
-        <f t="shared" si="6"/>
+      <c r="T24">
+        <f>ROUND(R24*0.033+Q57+S24, 2)</f>
         <v>0.5</v>
       </c>
-      <c r="U24">
-        <f t="shared" si="2"/>
+      <c r="V24">
+        <f t="shared" si="1"/>
         <v>0.61650000000000005</v>
       </c>
-      <c r="V24">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="W24">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>65</v>
       </c>
@@ -2120,36 +2146,36 @@
       <c r="J25">
         <v>100</v>
       </c>
-      <c r="M25">
+      <c r="N25">
         <v>1000</v>
       </c>
-      <c r="N25">
-        <f t="shared" si="0"/>
-        <v>-12.366666666666665</v>
-      </c>
-      <c r="P25">
+      <c r="O25">
+        <f>C25-D25*20-E25*0.8-F25*0.6-H25*10+I25*15+J25/200-M25*5</f>
+        <v>-11.799999999999999</v>
+      </c>
+      <c r="Q25">
         <v>0.04</v>
       </c>
-      <c r="Q25">
+      <c r="R25">
         <v>16.5</v>
       </c>
-      <c r="R25">
+      <c r="S25">
         <v>0.05</v>
       </c>
-      <c r="S25">
-        <f t="shared" si="6"/>
+      <c r="T25">
+        <f>ROUND(R25*0.033+Q58+S25, 2)</f>
         <v>0.59</v>
       </c>
-      <c r="U25">
-        <f t="shared" si="2"/>
+      <c r="V25">
+        <f t="shared" si="1"/>
         <v>0.72049999999999992</v>
       </c>
-      <c r="V25">
-        <f t="shared" si="3"/>
+      <c r="W25">
+        <f t="shared" si="2"/>
         <v>-8.5999999999999993E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>67</v>
       </c>
@@ -2177,36 +2203,36 @@
       <c r="J26">
         <v>100</v>
       </c>
-      <c r="M26">
+      <c r="N26">
         <v>1000</v>
       </c>
-      <c r="N26">
-        <f t="shared" si="0"/>
-        <v>-11.666666666666664</v>
-      </c>
-      <c r="P26">
+      <c r="O26">
+        <f>C26-D26*20-E26*0.8-F26*0.6-H26*10+I26*15+J26/200-M26*5</f>
+        <v>-10.999999999999998</v>
+      </c>
+      <c r="Q26">
         <v>0.04</v>
       </c>
-      <c r="Q26">
+      <c r="R26">
         <v>16.5</v>
       </c>
-      <c r="R26">
+      <c r="S26">
         <v>0.02</v>
       </c>
-      <c r="S26">
-        <f t="shared" si="6"/>
+      <c r="T26">
+        <f>ROUND(R26*0.033+Q59+S26, 2)</f>
         <v>0.56000000000000005</v>
       </c>
-      <c r="U26">
-        <f t="shared" si="2"/>
+      <c r="V26">
+        <f t="shared" si="1"/>
         <v>0.69049999999999989</v>
       </c>
-      <c r="V26">
-        <f t="shared" si="3"/>
+      <c r="W26">
+        <f t="shared" si="2"/>
         <v>-8.5999999999999993E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>69</v>
       </c>
@@ -2234,36 +2260,36 @@
       <c r="J27">
         <v>190</v>
       </c>
-      <c r="M27">
+      <c r="N27">
         <v>2000</v>
       </c>
-      <c r="N27">
-        <f t="shared" si="0"/>
-        <v>-12.116666666666667</v>
-      </c>
-      <c r="P27">
+      <c r="O27">
+        <f>C27-D27*20-E27*0.8-F27*0.6-H27*10+I27*15+J27/200-M27*5</f>
+        <v>-10.700000000000001</v>
+      </c>
+      <c r="Q27">
         <v>0.04</v>
       </c>
-      <c r="Q27">
+      <c r="R27">
         <v>20</v>
       </c>
-      <c r="R27">
+      <c r="S27">
         <v>0.05</v>
       </c>
-      <c r="S27">
-        <f t="shared" si="6"/>
+      <c r="T27">
+        <f>ROUND(R27*0.033+Q60+S27, 2)</f>
         <v>0.71</v>
       </c>
-      <c r="U27">
-        <f t="shared" si="2"/>
+      <c r="V27">
+        <f t="shared" si="1"/>
         <v>0.85000000000000009</v>
       </c>
-      <c r="V27">
-        <f t="shared" si="3"/>
+      <c r="W27">
+        <f t="shared" si="2"/>
         <v>-0.23649999999999999</v>
       </c>
     </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>71</v>
       </c>
@@ -2291,36 +2317,36 @@
       <c r="J28">
         <v>190</v>
       </c>
-      <c r="M28">
+      <c r="N28">
         <v>2000</v>
       </c>
-      <c r="N28">
-        <f t="shared" si="0"/>
-        <v>-11.416666666666666</v>
-      </c>
-      <c r="P28">
+      <c r="O28">
+        <f>C28-D28*20-E28*0.8-F28*0.6-H28*10+I28*15+J28/200-M28*5</f>
+        <v>-9.8999999999999986</v>
+      </c>
+      <c r="Q28">
         <v>0.04</v>
       </c>
-      <c r="Q28">
+      <c r="R28">
         <v>20</v>
       </c>
-      <c r="R28">
+      <c r="S28">
         <v>0.02</v>
       </c>
-      <c r="S28">
-        <f t="shared" si="6"/>
+      <c r="T28">
+        <f>ROUND(R28*0.033+Q61+S28, 2)</f>
         <v>0.68</v>
       </c>
-      <c r="U28">
-        <f t="shared" si="2"/>
+      <c r="V28">
+        <f t="shared" si="1"/>
         <v>0.82000000000000006</v>
       </c>
-      <c r="V28">
-        <f t="shared" si="3"/>
+      <c r="W28">
+        <f t="shared" si="2"/>
         <v>-0.23649999999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -2334,29 +2360,26 @@
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
-      <c r="N29">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="S29">
-        <f t="shared" ref="S29:S39" si="7">ROUND(Q29*0.033+P29+R29, 2)</f>
-        <v>0</v>
-      </c>
-      <c r="U29">
-        <f t="shared" si="2"/>
+      <c r="N29" s="1"/>
+      <c r="T29">
+        <f t="shared" ref="T29:T43" si="5">ROUND(R29*0.033+Q29+S29, 2)</f>
+        <v>0</v>
+      </c>
+      <c r="V29">
+        <f t="shared" si="1"/>
         <v>0.06</v>
       </c>
-      <c r="V29">
-        <f t="shared" si="3"/>
+      <c r="W29">
+        <f t="shared" si="2"/>
         <v>0.62349999999999994</v>
       </c>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>73</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="C30" s="1">
         <v>-8</v>
@@ -2382,41 +2405,42 @@
       </c>
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
-      <c r="M30" s="1">
+      <c r="M30" s="1"/>
+      <c r="N30" s="1">
         <v>2000</v>
       </c>
-      <c r="N30">
-        <f t="shared" si="0"/>
-        <v>-9.7533333333333321</v>
-      </c>
-      <c r="P30">
+      <c r="O30">
+        <f>C30-D30*20-E30*0.8-F30*0.6-H30*10+I30*15+J30/200-M30*5</f>
+        <v>-8.7049999999999983</v>
+      </c>
+      <c r="Q30">
         <v>0.1</v>
       </c>
-      <c r="Q30">
+      <c r="R30">
         <v>24.409400000000002</v>
       </c>
-      <c r="R30">
+      <c r="S30">
         <v>0.1</v>
       </c>
-      <c r="S30">
-        <f t="shared" si="7"/>
+      <c r="T30">
+        <f t="shared" si="5"/>
         <v>1.01</v>
       </c>
-      <c r="U30">
-        <f t="shared" si="2"/>
+      <c r="V30">
+        <f t="shared" si="1"/>
         <v>1.0631478000000001</v>
       </c>
-      <c r="V30">
-        <f t="shared" si="3"/>
+      <c r="W30">
+        <f t="shared" si="2"/>
         <v>-0.42610420000000004</v>
       </c>
     </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
+      </c>
+      <c r="B31" t="s">
+        <v>93</v>
       </c>
       <c r="C31" s="1">
         <v>-4</v>
@@ -2442,38 +2466,39 @@
       </c>
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
-      <c r="M31" s="1">
+      <c r="M31" s="1"/>
+      <c r="N31" s="1">
         <v>1000</v>
       </c>
-      <c r="N31">
-        <f t="shared" si="0"/>
-        <v>-8.0533333333333346</v>
-      </c>
-      <c r="P31">
+      <c r="O31">
+        <f>C31-D31*20-E31*0.8-F31*0.6-H31*10+I31*15+J31/200-M31*5</f>
+        <v>-6.5549999999999997</v>
+      </c>
+      <c r="Q31">
         <v>0.1</v>
       </c>
-      <c r="Q31">
+      <c r="R31">
         <v>20</v>
       </c>
-      <c r="S31">
-        <f t="shared" si="7"/>
+      <c r="T31">
+        <f t="shared" si="5"/>
         <v>0.76</v>
       </c>
-      <c r="U31">
-        <f t="shared" si="2"/>
+      <c r="V31">
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
-      <c r="V31">
-        <f t="shared" si="3"/>
+      <c r="W31">
+        <f t="shared" si="2"/>
         <v>-0.23649999999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>78</v>
+        <v>75</v>
+      </c>
+      <c r="B32" t="s">
+        <v>94</v>
       </c>
       <c r="C32" s="1">
         <v>-2</v>
@@ -2499,38 +2524,39 @@
       </c>
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
-      <c r="M32" s="1">
+      <c r="M32" s="1"/>
+      <c r="N32" s="1">
         <v>750</v>
       </c>
-      <c r="N32">
-        <f t="shared" si="0"/>
-        <v>-8.7633333333333319</v>
-      </c>
-      <c r="P32">
+      <c r="O32">
+        <f>C32-D32*20-E32*0.8-F32*0.6-H32*10+I32*15+J32/200-M32*5</f>
+        <v>-7.794999999999999</v>
+      </c>
+      <c r="Q32">
         <v>0.1</v>
       </c>
-      <c r="Q32">
+      <c r="R32">
         <v>17.992100000000001</v>
       </c>
-      <c r="S32">
-        <f t="shared" si="7"/>
+      <c r="T32">
+        <f t="shared" si="5"/>
         <v>0.69</v>
       </c>
-      <c r="U32">
-        <f t="shared" si="2"/>
+      <c r="V32">
+        <f t="shared" si="1"/>
         <v>0.72570770000000007</v>
       </c>
-      <c r="V32">
-        <f t="shared" si="3"/>
+      <c r="W32">
+        <f t="shared" si="2"/>
         <v>-0.15016030000000002</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
+      </c>
+      <c r="B33" t="s">
+        <v>95</v>
       </c>
       <c r="C33" s="1">
         <v>0</v>
@@ -2556,38 +2582,39 @@
       </c>
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
-      <c r="M33" s="1">
-        <v>0</v>
-      </c>
-      <c r="N33">
-        <f t="shared" si="0"/>
-        <v>-9.5366666666666653</v>
-      </c>
-      <c r="P33">
+      <c r="M33" s="1"/>
+      <c r="N33" s="1">
+        <v>0</v>
+      </c>
+      <c r="O33">
+        <f>C33-D33*20-E33*0.8-F33*0.6-H33*10+I33*15+J33/200-M33*5</f>
+        <v>-9.1050000000000004</v>
+      </c>
+      <c r="Q33">
         <v>0.1</v>
       </c>
-      <c r="Q33">
+      <c r="R33">
         <v>16.023599999999998</v>
       </c>
-      <c r="S33">
-        <f t="shared" si="7"/>
+      <c r="T33">
+        <f t="shared" si="5"/>
         <v>0.63</v>
       </c>
-      <c r="U33">
-        <f t="shared" si="2"/>
+      <c r="V33">
+        <f t="shared" si="1"/>
         <v>0.65287319999999993</v>
       </c>
-      <c r="V33">
-        <f t="shared" si="3"/>
+      <c r="W33">
+        <f t="shared" si="2"/>
         <v>-6.5514799999999915E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>82</v>
+        <v>77</v>
+      </c>
+      <c r="B34" t="s">
+        <v>96</v>
       </c>
       <c r="C34" s="1">
         <v>2</v>
@@ -2613,235 +2640,178 @@
       </c>
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
-      <c r="M34" s="1">
+      <c r="M34" s="1"/>
+      <c r="N34" s="1">
         <v>600</v>
       </c>
-      <c r="N34">
-        <f t="shared" si="0"/>
-        <v>-9.3666666666666654</v>
-      </c>
-      <c r="P34">
+      <c r="O34">
+        <f>C34-D34*20-E34*0.8-F34*0.6-H34*10+I34*15+J34/200-M34*5</f>
+        <v>-9.4999999999999982</v>
+      </c>
+      <c r="Q34">
         <v>0.1</v>
       </c>
-      <c r="Q34">
+      <c r="R34">
         <v>13.779500000000001</v>
       </c>
-      <c r="S34">
-        <f t="shared" si="7"/>
+      <c r="T34">
+        <f t="shared" si="5"/>
         <v>0.55000000000000004</v>
       </c>
-      <c r="U34">
-        <f t="shared" si="2"/>
+      <c r="V34">
+        <f t="shared" si="1"/>
         <v>0.56984149999999989</v>
       </c>
-      <c r="V34">
-        <f t="shared" si="3"/>
+      <c r="W34">
+        <f t="shared" si="2"/>
         <v>3.0981499999999974E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A35" s="1"/>
-      <c r="B35" s="1"/>
-      <c r="C35" s="1"/>
-      <c r="D35" s="1"/>
-      <c r="E35" s="1"/>
-      <c r="F35" s="1"/>
-      <c r="G35" s="1"/>
-      <c r="H35" s="1"/>
-      <c r="I35" s="1"/>
-      <c r="J35" s="1"/>
-      <c r="K35" s="1"/>
-      <c r="L35" s="1"/>
-      <c r="M35" s="1"/>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>84</v>
+      </c>
+      <c r="B35" t="s">
+        <v>85</v>
+      </c>
+      <c r="C35">
+        <v>2</v>
+      </c>
+      <c r="D35">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
+      </c>
+      <c r="H35">
+        <v>0.08</v>
+      </c>
+      <c r="I35">
+        <v>0.01</v>
+      </c>
+      <c r="J35">
+        <v>10</v>
+      </c>
       <c r="N35">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="S35">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="U35">
-        <f t="shared" si="2"/>
-        <v>0.06</v>
-      </c>
-      <c r="V35">
-        <f t="shared" si="3"/>
-        <v>0.62349999999999994</v>
-      </c>
-    </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="C36" s="1">
+        <v>2100</v>
+      </c>
+      <c r="O35">
+        <f t="shared" ref="O35:O38" si="6">C35-D35*20-E35*0.8-F35*0.6-H35*10+I35*15+J35/200-M35*5</f>
+        <v>-9.9999999999999982</v>
+      </c>
+    </row>
+    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>86</v>
+      </c>
+      <c r="B36" t="s">
+        <v>87</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <v>0.65</v>
+      </c>
+      <c r="E36">
+        <v>-1</v>
+      </c>
+      <c r="F36">
+        <v>-1</v>
+      </c>
+      <c r="H36">
+        <v>-0.01</v>
+      </c>
+      <c r="I36">
+        <v>0.1</v>
+      </c>
+      <c r="J36">
+        <v>79</v>
+      </c>
+      <c r="N36">
+        <v>1500</v>
+      </c>
+      <c r="O36">
+        <f t="shared" si="6"/>
+        <v>-9.6050000000000004</v>
+      </c>
+    </row>
+    <row r="37" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>88</v>
+      </c>
+      <c r="B37" t="s">
+        <v>89</v>
+      </c>
+      <c r="C37">
+        <v>-2</v>
+      </c>
+      <c r="D37">
+        <v>0.72</v>
+      </c>
+      <c r="E37">
+        <v>-3</v>
+      </c>
+      <c r="F37">
+        <v>-3</v>
+      </c>
+      <c r="H37">
+        <v>-0.1</v>
+      </c>
+      <c r="I37">
+        <v>0.15</v>
+      </c>
+      <c r="J37">
+        <v>131</v>
+      </c>
+      <c r="N37">
+        <v>2250</v>
+      </c>
+      <c r="O37">
+        <f t="shared" si="6"/>
+        <v>-8.2949999999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>90</v>
+      </c>
+      <c r="B38" t="s">
+        <v>91</v>
+      </c>
+      <c r="C38">
+        <v>-4</v>
+      </c>
+      <c r="D38">
+        <v>0.8</v>
+      </c>
+      <c r="E38">
         <v>-5</v>
       </c>
-      <c r="D36" s="1">
-        <v>0.73</v>
-      </c>
-      <c r="E36" s="1">
-        <v>-4</v>
-      </c>
-      <c r="F36" s="1">
-        <v>-4</v>
-      </c>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1">
-        <v>-0.13</v>
-      </c>
-      <c r="I36" s="1">
-        <v>0.16</v>
-      </c>
-      <c r="J36" s="1">
-        <v>131</v>
-      </c>
-      <c r="K36" s="1"/>
-      <c r="L36" s="1"/>
-      <c r="M36" s="1">
-        <v>1500</v>
-      </c>
-      <c r="N36">
-        <f t="shared" si="0"/>
-        <v>-10.513333333333334</v>
-      </c>
-      <c r="P36">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="Q36">
-        <v>17.992100000000001</v>
-      </c>
-      <c r="S36">
-        <f t="shared" si="7"/>
-        <v>0.73</v>
-      </c>
-      <c r="U36">
-        <f t="shared" si="2"/>
-        <v>0.72570770000000007</v>
-      </c>
-      <c r="V36">
-        <f t="shared" si="3"/>
-        <v>-0.15016030000000002</v>
-      </c>
-    </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C37" s="1">
-        <v>0</v>
-      </c>
-      <c r="D37" s="1">
-        <v>0.6</v>
-      </c>
-      <c r="E37" s="1">
-        <v>0</v>
-      </c>
-      <c r="F37" s="1">
-        <v>0</v>
-      </c>
-      <c r="G37" s="1"/>
-      <c r="H37" s="1">
-        <v>0.04</v>
-      </c>
-      <c r="I37" s="1">
-        <v>0.02</v>
-      </c>
-      <c r="J37" s="1">
-        <v>17</v>
-      </c>
-      <c r="K37" s="1"/>
-      <c r="L37" s="1"/>
-      <c r="M37" s="1">
-        <v>0</v>
-      </c>
-      <c r="N37">
-        <f t="shared" si="0"/>
-        <v>-11.843333333333332</v>
-      </c>
-      <c r="P37">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="Q37">
-        <v>13.9764</v>
-      </c>
-      <c r="S37">
-        <f t="shared" si="7"/>
-        <v>0.6</v>
-      </c>
-      <c r="U37">
-        <f t="shared" si="2"/>
-        <v>0.57712680000000005</v>
-      </c>
-      <c r="V37">
-        <f t="shared" si="3"/>
-        <v>2.2514800000000001E-2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C38" s="1">
-        <v>2</v>
-      </c>
-      <c r="D38" s="1">
-        <v>0.47</v>
-      </c>
-      <c r="E38" s="1">
-        <v>1</v>
-      </c>
-      <c r="F38" s="1">
-        <v>1</v>
-      </c>
-      <c r="G38" s="1"/>
-      <c r="H38" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="I38" s="1">
-        <v>-0.08</v>
-      </c>
-      <c r="J38" s="1">
-        <v>-135</v>
-      </c>
-      <c r="K38" s="1"/>
-      <c r="L38" s="1"/>
-      <c r="M38" s="1">
-        <v>1200</v>
+      <c r="F38">
+        <v>-5</v>
+      </c>
+      <c r="H38">
+        <v>-0.19</v>
+      </c>
+      <c r="I38">
+        <v>0.21</v>
+      </c>
+      <c r="J38">
+        <v>179</v>
       </c>
       <c r="N38">
-        <f t="shared" si="0"/>
-        <v>-11.449999999999998</v>
-      </c>
-      <c r="P38">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="Q38">
-        <v>10</v>
-      </c>
-      <c r="S38">
-        <f t="shared" si="7"/>
-        <v>0.47</v>
-      </c>
-      <c r="U38">
-        <f t="shared" si="2"/>
-        <v>0.43</v>
-      </c>
-      <c r="V38">
-        <f t="shared" si="3"/>
-        <v>0.19349999999999998</v>
-      </c>
-    </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
+        <v>2500</v>
+      </c>
+      <c r="O38">
+        <f t="shared" si="6"/>
+        <v>-7.0549999999999997</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -2855,61 +2825,199 @@
       <c r="K39" s="1"/>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
-      <c r="N39">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="S39">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A40" s="1"/>
-      <c r="B40" s="1"/>
-      <c r="C40" s="1"/>
-      <c r="D40" s="1"/>
-      <c r="E40" s="1"/>
-      <c r="F40" s="1"/>
+      <c r="N39" s="1"/>
+      <c r="O39">
+        <f>C39-D39*20-E39*0.8-F39*0.6-H39*5+I39*15+J39/300</f>
+        <v>0</v>
+      </c>
+      <c r="T39">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="V39">
+        <f t="shared" si="1"/>
+        <v>0.06</v>
+      </c>
+      <c r="W39">
+        <f t="shared" si="2"/>
+        <v>0.62349999999999994</v>
+      </c>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C40" s="1">
+        <v>-5</v>
+      </c>
+      <c r="D40" s="1">
+        <v>0.73</v>
+      </c>
+      <c r="E40" s="1">
+        <v>-4</v>
+      </c>
+      <c r="F40" s="1">
+        <v>-4</v>
+      </c>
       <c r="G40" s="1"/>
-      <c r="H40" s="1"/>
-      <c r="I40" s="1"/>
-      <c r="J40" s="1"/>
+      <c r="H40" s="1">
+        <v>-0.13</v>
+      </c>
+      <c r="I40" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="J40" s="1">
+        <v>131</v>
+      </c>
       <c r="K40" s="1"/>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
-    </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A41" s="1"/>
-      <c r="B41" s="1"/>
-      <c r="C41" s="1"/>
-      <c r="D41" s="1"/>
-      <c r="E41" s="1"/>
-      <c r="F41" s="1"/>
+      <c r="N40" s="1">
+        <v>1500</v>
+      </c>
+      <c r="O40">
+        <f>C40-D40*20-E40*0.8-F40*0.6-H40*5+I40*15+J40/300</f>
+        <v>-10.513333333333334</v>
+      </c>
+      <c r="Q40">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="R40">
+        <v>17.992100000000001</v>
+      </c>
+      <c r="T40">
+        <f t="shared" si="5"/>
+        <v>0.73</v>
+      </c>
+      <c r="V40">
+        <f t="shared" si="1"/>
+        <v>0.72570770000000007</v>
+      </c>
+      <c r="W40">
+        <f t="shared" si="2"/>
+        <v>-0.15016030000000002</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C41" s="1">
+        <v>0</v>
+      </c>
+      <c r="D41" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="E41" s="1">
+        <v>0</v>
+      </c>
+      <c r="F41" s="1">
+        <v>0</v>
+      </c>
       <c r="G41" s="1"/>
-      <c r="H41" s="1"/>
-      <c r="I41" s="1"/>
-      <c r="J41" s="1"/>
+      <c r="H41" s="1">
+        <v>0.04</v>
+      </c>
+      <c r="I41" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="J41" s="1">
+        <v>17</v>
+      </c>
       <c r="K41" s="1"/>
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
-    </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A42" s="1"/>
-      <c r="B42" s="1"/>
-      <c r="C42" s="1"/>
-      <c r="D42" s="1"/>
-      <c r="E42" s="1"/>
-      <c r="F42" s="1"/>
+      <c r="N41" s="1">
+        <v>0</v>
+      </c>
+      <c r="O41">
+        <f>C41-D41*20-E41*0.8-F41*0.6-H41*5+I41*15+J41/300</f>
+        <v>-11.843333333333332</v>
+      </c>
+      <c r="Q41">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="R41">
+        <v>13.9764</v>
+      </c>
+      <c r="T41">
+        <f t="shared" si="5"/>
+        <v>0.6</v>
+      </c>
+      <c r="V41">
+        <f t="shared" si="1"/>
+        <v>0.57712680000000005</v>
+      </c>
+      <c r="W41">
+        <f t="shared" si="2"/>
+        <v>2.2514800000000001E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C42" s="1">
+        <v>2</v>
+      </c>
+      <c r="D42" s="1">
+        <v>0.47</v>
+      </c>
+      <c r="E42" s="1">
+        <v>1</v>
+      </c>
+      <c r="F42" s="1">
+        <v>1</v>
+      </c>
       <c r="G42" s="1"/>
-      <c r="H42" s="1"/>
-      <c r="I42" s="1"/>
-      <c r="J42" s="1"/>
+      <c r="H42" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="I42" s="1">
+        <v>-0.08</v>
+      </c>
+      <c r="J42" s="1">
+        <v>-135</v>
+      </c>
       <c r="K42" s="1"/>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
-    </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="N42" s="1">
+        <v>1200</v>
+      </c>
+      <c r="O42">
+        <f>C42-D42*20-E42*0.8-F42*0.6-H42*5+I42*15+J42/300</f>
+        <v>-11.449999999999998</v>
+      </c>
+      <c r="Q42">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="R42">
+        <v>10</v>
+      </c>
+      <c r="T42">
+        <f t="shared" si="5"/>
+        <v>0.47</v>
+      </c>
+      <c r="V42">
+        <f t="shared" si="1"/>
+        <v>0.43</v>
+      </c>
+      <c r="W42">
+        <f t="shared" si="2"/>
+        <v>0.19349999999999998</v>
+      </c>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -2923,8 +3031,17 @@
       <c r="K43" s="1"/>
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
-    </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="N43" s="1"/>
+      <c r="O43">
+        <f>C43-D43*20-E43*0.8-F43*0.6-H43*5+I43*15+J43/300</f>
+        <v>0</v>
+      </c>
+      <c r="T43">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -2938,8 +3055,9 @@
       <c r="K44" s="1"/>
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
-    </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="N44" s="1"/>
+    </row>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -2953,8 +3071,9 @@
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
       <c r="M45" s="1"/>
-    </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="N45" s="1"/>
+    </row>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -2968,6 +3087,71 @@
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
       <c r="M46" s="1"/>
+      <c r="N46" s="1"/>
+    </row>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A47" s="1"/>
+      <c r="B47" s="1"/>
+      <c r="C47" s="1"/>
+      <c r="D47" s="1"/>
+      <c r="E47" s="1"/>
+      <c r="F47" s="1"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="1"/>
+      <c r="I47" s="1"/>
+      <c r="J47" s="1"/>
+      <c r="K47" s="1"/>
+      <c r="L47" s="1"/>
+      <c r="M47" s="1"/>
+      <c r="N47" s="1"/>
+    </row>
+    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A48" s="1"/>
+      <c r="B48" s="1"/>
+      <c r="C48" s="1"/>
+      <c r="D48" s="1"/>
+      <c r="E48" s="1"/>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
+      <c r="I48" s="1"/>
+      <c r="J48" s="1"/>
+      <c r="K48" s="1"/>
+      <c r="L48" s="1"/>
+      <c r="M48" s="1"/>
+      <c r="N48" s="1"/>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A49" s="1"/>
+      <c r="B49" s="1"/>
+      <c r="C49" s="1"/>
+      <c r="D49" s="1"/>
+      <c r="E49" s="1"/>
+      <c r="F49" s="1"/>
+      <c r="G49" s="1"/>
+      <c r="H49" s="1"/>
+      <c r="I49" s="1"/>
+      <c r="J49" s="1"/>
+      <c r="K49" s="1"/>
+      <c r="L49" s="1"/>
+      <c r="M49" s="1"/>
+      <c r="N49" s="1"/>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A50" s="1"/>
+      <c r="B50" s="1"/>
+      <c r="C50" s="1"/>
+      <c r="D50" s="1"/>
+      <c r="E50" s="1"/>
+      <c r="F50" s="1"/>
+      <c r="G50" s="1"/>
+      <c r="H50" s="1"/>
+      <c r="I50" s="1"/>
+      <c r="J50" s="1"/>
+      <c r="K50" s="1"/>
+      <c r="L50" s="1"/>
+      <c r="M50" s="1"/>
+      <c r="N50" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>